<commit_message>
Re-doing: discovered a woopsie in the plating nrs
</commit_message>
<xml_diff>
--- a/Cell survival results/Analysis Corrected results 16 Oct/Proton high.xlsx
+++ b/Cell survival results/Analysis Corrected results 16 Oct/Proton high.xlsx
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7494.4</v>
+        <v>2810.4</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14988.8</v>
+        <v>5620.8</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>

</xml_diff>